<commit_message>
Modified metrics and analysis for all partecipants
</commit_message>
<xml_diff>
--- a/questionari/risposte/Edinburgh Test Hand Dominance - VISIONARY (Responses).xlsx
+++ b/questionari/risposte/Edinburgh Test Hand Dominance - VISIONARY (Responses).xlsx
@@ -201,7 +201,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Form_Responses" displayName="Form_Responses" ref="A1:L7" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Form_Responses" displayName="Form_Responses" ref="A1:L12" headerRowCount="1">
   <tableColumns count="12">
     <tableColumn id="1" name="Timestamp"/>
     <tableColumn id="2" name="ID"/>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="18.88" customWidth="1" style="6" min="1" max="7"/>
@@ -854,7 +854,306 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="22.5" customHeight="1" s="6"/>
+    <row r="8" ht="22.5" customHeight="1" s="6">
+      <c r="A8" s="4" t="n">
+        <v>46296.43380547454</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>S007</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Right hand (strong preference)</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Right hand (strong preference)</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Right hand</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Right hand</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Indifferent/Both</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Right hand</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Indifferent/Both</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Right hand</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Right hand (strong preference)</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Indifferent/Both</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22.5" customHeight="1" s="6">
+      <c r="A9" s="4" t="n">
+        <v>46296.49612587963</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>S008</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Right hand</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Right hand</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Right hand</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Right hand</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Right hand</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Left hand</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Right hand</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Right hand</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>Right hand</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>Right hand</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22.5" customHeight="1" s="6">
+      <c r="A10" s="4" t="n">
+        <v>46296.58566054398</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>S009</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Right hand (strong preference)</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Right hand (strong preference)</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Right hand</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Right hand (strong preference)</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Right hand (strong preference)</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Right hand (strong preference)</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Right hand (strong preference)</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Right hand (strong preference)</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>Right hand (strong preference)</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Right hand (strong preference)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22.5" customHeight="1" s="6">
+      <c r="A11" s="4" t="n">
+        <v>46296.64122185185</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>S010</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Right hand (strong preference)</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Right hand (strong preference)</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Right hand (strong preference)</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Right hand (strong preference)</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Right hand (strong preference)</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Right hand (strong preference)</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Right hand (strong preference)</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Right hand (strong preference)</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>Right hand (strong preference)</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>Right hand (strong preference)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22.5" customHeight="1" s="6">
+      <c r="A12" s="4" t="n">
+        <v>46296.6905272338</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>S011</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Left hand (strong preference)</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Left hand (strong preference)</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Right hand (strong preference)</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Right hand</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Right hand</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Right hand</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Right hand</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>Indifferent/Both</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>Right hand</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>Indifferent/Both</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Removed S007 and modified some analysis
</commit_message>
<xml_diff>
--- a/questionari/risposte/Edinburgh Test Hand Dominance - VISIONARY (Responses).xlsx
+++ b/questionari/risposte/Edinburgh Test Hand Dominance - VISIONARY (Responses).xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="18.88" customWidth="1" style="6" min="1" max="7"/>
@@ -856,7 +856,7 @@
     </row>
     <row r="8" ht="22.5" customHeight="1" s="6">
       <c r="A8" s="4" t="n">
-        <v>46296.43380547454</v>
+        <v>46296.49612587963</v>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
@@ -865,12 +865,12 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Right hand (strong preference)</t>
+          <t>Right hand</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Right hand (strong preference)</t>
+          <t>Right hand</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -885,17 +885,17 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Indifferent/Both</t>
+          <t>Right hand</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Right hand</t>
+          <t>Left hand</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Indifferent/Both</t>
+          <t>Right hand</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
@@ -905,18 +905,18 @@
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>Right hand (strong preference)</t>
+          <t>Right hand</t>
         </is>
       </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>Indifferent/Both</t>
+          <t>Right hand</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1" s="6">
       <c r="A9" s="4" t="n">
-        <v>46296.49612587963</v>
+        <v>46296.58566054398</v>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
@@ -925,12 +925,12 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Right hand</t>
+          <t>Right hand (strong preference)</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Right hand</t>
+          <t>Right hand (strong preference)</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -940,43 +940,43 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Right hand</t>
+          <t>Right hand (strong preference)</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Right hand</t>
+          <t>Right hand (strong preference)</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Left hand</t>
+          <t>Right hand (strong preference)</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Right hand</t>
+          <t>Right hand (strong preference)</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Right hand</t>
+          <t>Right hand (strong preference)</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>Right hand</t>
+          <t>Right hand (strong preference)</t>
         </is>
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>Right hand</t>
+          <t>Right hand (strong preference)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1" s="6">
       <c r="A10" s="4" t="n">
-        <v>46296.58566054398</v>
+        <v>46296.64122185185</v>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
@@ -995,7 +995,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Right hand</t>
+          <t>Right hand (strong preference)</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -1036,7 +1036,7 @@
     </row>
     <row r="11" ht="22.5" customHeight="1" s="6">
       <c r="A11" s="4" t="n">
-        <v>46296.64122185185</v>
+        <v>46296.6905272338</v>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
@@ -1045,12 +1045,12 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Right hand (strong preference)</t>
+          <t>Left hand (strong preference)</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Right hand (strong preference)</t>
+          <t>Left hand (strong preference)</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -1060,100 +1060,41 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Right hand (strong preference)</t>
+          <t>Right hand</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Right hand (strong preference)</t>
+          <t>Right hand</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Right hand (strong preference)</t>
+          <t>Right hand</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Right hand (strong preference)</t>
+          <t>Right hand</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>Right hand (strong preference)</t>
+          <t>Indifferent/Both</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
-          <t>Right hand (strong preference)</t>
+          <t>Right hand</t>
         </is>
       </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>Right hand (strong preference)</t>
+          <t>Indifferent/Both</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="22.5" customHeight="1" s="6">
-      <c r="A12" s="4" t="n">
-        <v>46296.6905272338</v>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>S011</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Left hand (strong preference)</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Left hand (strong preference)</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Right hand (strong preference)</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>Right hand</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>Right hand</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>Right hand</t>
-        </is>
-      </c>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>Right hand</t>
-        </is>
-      </c>
-      <c r="J12" s="5" t="inlineStr">
-        <is>
-          <t>Indifferent/Both</t>
-        </is>
-      </c>
-      <c r="K12" s="5" t="inlineStr">
-        <is>
-          <t>Right hand</t>
-        </is>
-      </c>
-      <c r="L12" s="5" t="inlineStr">
-        <is>
-          <t>Indifferent/Both</t>
-        </is>
-      </c>
-    </row>
+    <row r="12" ht="22.5" customHeight="1" s="6"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>